<commit_message>
recipes: rescue second intake review recipes
</commit_message>
<xml_diff>
--- a/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
+++ b/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="1" r:id="R5099330131534377"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ingredients" sheetId="2" r:id="Re595dd23bd5e4fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="steps" sheetId="3" r:id="Reb65626261544c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qa_issues" sheetId="4" r:id="R3034eba3a94d4b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="1" r:id="R2ced93ef012f4016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ingredients" sheetId="2" r:id="R35bd9e57f9964832"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="steps" sheetId="3" r:id="R1f339bfb8d7a4f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qa_issues" sheetId="4" r:id="R849963b25abb4532"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -627,7 +627,7 @@
         <x:v>Фотореалистичное фото: онигири, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R3" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" hidden="0" customHeight="1">
@@ -795,7 +795,7 @@
         <x:v>Фотореалистичное фото: рулет из лаваша с крабовыми палочками, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R6" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" hidden="0" customHeight="1">
@@ -3427,7 +3427,7 @@
         <x:v>Фотореалистичное фото: картофельные ньокки, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R53" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="36" hidden="0" customHeight="1">
@@ -3483,7 +3483,7 @@
         <x:v>Фотореалистичное фото: пицца на основе из цветной капусты, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R54" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="36" hidden="0" customHeight="1">
@@ -3595,7 +3595,7 @@
         <x:v>Фотореалистичное фото: рулетики из баклажанов с мясом и сыром, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R56" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="36" hidden="0" customHeight="1">
@@ -3875,7 +3875,7 @@
         <x:v>Фотореалистичное фото: энчилада в кукурузных тортильях, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R61" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="36" hidden="0" customHeight="1">
@@ -6227,7 +6227,7 @@
         <x:v>Фотореалистичное фото: ленивая пицца на лаваше, одна порция, естественный дневной свет, нейтральная тарелка, аккуратная подача, без текста и упаковок.</x:v>
       </x:c>
       <x:c r="R103" s="25" t="str">
-        <x:v>needs_review</x:v>
+        <x:v>ready</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="36" hidden="0" customHeight="1">
@@ -6691,9 +6691,11 @@
       </x:c>
       <x:c r="F10" s="24" t="str"/>
       <x:c r="G10" s="24" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="H10" s="25" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="H10" s="25" t="str">
+        <x:v>Rescue policy: крабовые палочки поддержаны canonical food_id crab_sticks; не декомпозировать.</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="23" t="str">
@@ -7076,7 +7078,7 @@
         <x:v>batch2_005</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>плавленый сыр</x:v>
+        <x:v>творожный сыр</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
         <x:v>1</x:v>
@@ -7091,7 +7093,9 @@
       <x:c r="G28" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="H28" s="25" t="str"/>
+      <x:c r="H28" s="25" t="str">
+        <x:v>Rescue policy: плавленый сыр заменен на творожный сыр; кулинарный смысл рулета сохранен.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="23" t="str">
@@ -7111,9 +7115,11 @@
       </x:c>
       <x:c r="F29" s="24" t="str"/>
       <x:c r="G29" s="24" t="str">
-        <x:v>no</x:v>
-      </x:c>
-      <x:c r="H29" s="25" t="str"/>
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="H29" s="25" t="str">
+        <x:v>Rescue policy: крабовые палочки поддержаны canonical food_id crab_sticks; не декомпозировать.</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="23" t="str">
@@ -15144,7 +15150,7 @@
         <x:v>batch2_052</x:v>
       </x:c>
       <x:c r="B382" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C382" s="24" t="str">
         <x:v>120</x:v>
@@ -15155,12 +15161,14 @@
       <x:c r="E382" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F382" s="24" t="str"/>
+      <x:c r="F382" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G382" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H382" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем.</x:v>
       </x:c>
     </x:row>
     <x:row r="383" ht="24" hidden="0" customHeight="1">
@@ -15264,7 +15272,7 @@
         <x:v>batch2_053</x:v>
       </x:c>
       <x:c r="B387" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C387" s="24" t="str">
         <x:v>120</x:v>
@@ -15275,12 +15283,14 @@
       <x:c r="E387" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F387" s="24" t="str"/>
+      <x:c r="F387" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G387" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H387" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем.</x:v>
       </x:c>
     </x:row>
     <x:row r="388" ht="24" hidden="0" customHeight="1">
@@ -15572,7 +15582,7 @@
         <x:v>batch2_055</x:v>
       </x:c>
       <x:c r="B400" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C400" s="24" t="str">
         <x:v>120</x:v>
@@ -15583,12 +15593,14 @@
       <x:c r="E400" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F400" s="24" t="str"/>
+      <x:c r="F400" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G400" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H400" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем.</x:v>
       </x:c>
     </x:row>
     <x:row r="401" ht="24" hidden="0" customHeight="1">
@@ -16417,7 +16429,7 @@
       </x:c>
       <x:c r="F435" s="24" t="str"/>
       <x:c r="G435" s="24" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="H435" s="25" t="str">
         <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
@@ -16452,7 +16464,7 @@
         <x:v>batch2_060</x:v>
       </x:c>
       <x:c r="B437" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C437" s="24" t="str">
         <x:v>120</x:v>
@@ -16463,12 +16475,14 @@
       <x:c r="E437" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F437" s="24" t="str"/>
+      <x:c r="F437" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G437" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H437" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем.</x:v>
       </x:c>
     </x:row>
     <x:row r="438" ht="24" hidden="0" customHeight="1">
@@ -16537,7 +16551,7 @@
       </x:c>
       <x:c r="F440" s="24" t="str"/>
       <x:c r="G440" s="24" t="str">
-        <x:v>yes</x:v>
+        <x:v>no</x:v>
       </x:c>
       <x:c r="H440" s="25" t="str">
         <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
@@ -19661,12 +19675,14 @@
       <x:c r="E573" s="24" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F573" s="24" t="str"/>
+      <x:c r="F573" s="24" t="str">
+        <x:v>масло слить, вес без масла</x:v>
+      </x:c>
       <x:c r="G573" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="H573" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Остается needs_review: в production foods нет canonical sprats/close canned fish mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="574" ht="24" hidden="0" customHeight="1">
@@ -19781,12 +19797,14 @@
       <x:c r="E578" s="24" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F578" s="24" t="str"/>
+      <x:c r="F578" s="24" t="str">
+        <x:v>масло слить, вес без масла</x:v>
+      </x:c>
       <x:c r="G578" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="H578" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Остается needs_review: в production foods нет canonical sprats/close canned fish mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="579" ht="24" hidden="0" customHeight="1">
@@ -19818,7 +19836,7 @@
         <x:v>batch2_084</x:v>
       </x:c>
       <x:c r="B580" s="24" t="str">
-        <x:v>уксус/лимонный сок</x:v>
+        <x:v>лимонный сок</x:v>
       </x:c>
       <x:c r="C580" s="24" t="str">
         <x:v>10</x:v>
@@ -19834,7 +19852,7 @@
         <x:v>no</x:v>
       </x:c>
       <x:c r="H580" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: optional vinegar/lemon row normalized to lemon juice used in the step.</x:v>
       </x:c>
     </x:row>
     <x:row r="581" ht="24" hidden="0" customHeight="1">
@@ -19923,12 +19941,14 @@
       <x:c r="E584" s="24" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F584" s="24" t="str"/>
+      <x:c r="F584" s="24" t="str">
+        <x:v>масло слить, вес без масла</x:v>
+      </x:c>
       <x:c r="G584" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="H584" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Остается needs_review: в production foods нет canonical sprats/close canned fish mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="585" ht="24" hidden="0" customHeight="1">
@@ -20041,12 +20061,14 @@
       <x:c r="E589" s="24" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F589" s="24" t="str"/>
+      <x:c r="F589" s="24" t="str">
+        <x:v>масло слить, вес без масла</x:v>
+      </x:c>
       <x:c r="G589" s="24" t="str">
         <x:v>yes</x:v>
       </x:c>
       <x:c r="H589" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Остается needs_review: в production foods нет canonical sprats/close canned fish mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="590" ht="24" hidden="0" customHeight="1">
@@ -21824,7 +21846,7 @@
         <x:v>batch2_102</x:v>
       </x:c>
       <x:c r="B666" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C666" s="24" t="str">
         <x:v>120</x:v>
@@ -21835,12 +21857,14 @@
       <x:c r="E666" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F666" s="24" t="str"/>
+      <x:c r="F666" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G666" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H666" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем.</x:v>
       </x:c>
     </x:row>
     <x:row r="667" ht="24" hidden="0" customHeight="1">
@@ -22240,7 +22264,7 @@
         <x:v>batch2_106</x:v>
       </x:c>
       <x:c r="B684" s="24" t="str">
-        <x:v>томатный соус</x:v>
+        <x:v>томаты в собственном соку</x:v>
       </x:c>
       <x:c r="C684" s="24" t="str">
         <x:v>120</x:v>
@@ -22251,12 +22275,14 @@
       <x:c r="E684" s="24" t="n">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="F684" s="24" t="str"/>
+      <x:c r="F684" s="24" t="str">
+        <x:v>без добавленного соуса</x:v>
+      </x:c>
       <x:c r="G684" s="24" t="str">
         <x:v>no</x:v>
       </x:c>
       <x:c r="H684" s="25" t="str">
-        <x:v>Количество восстановлено редакционно из названия/шага.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; рецепт остается needs_review из-за неточных source quantities.</x:v>
       </x:c>
     </x:row>
     <x:row r="685" ht="24" hidden="0" customHeight="1">
@@ -22496,7 +22522,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C14" s="25" t="str">
-        <x:v>Смажь лаваш йогуртом, выложи начинку и заверни тугой рулет, подвернув края снизу и сверху.</x:v>
+        <x:v>Смажь лаваш йогуртом и творожным сыром, выложи начинку и заверни тугой рулет, подвернув края снизу и сверху.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -23992,7 +24018,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C150" s="25" t="str">
-        <x:v>Подавай с томатным соусом и сыром.</x:v>
+        <x:v>Подавай с томатами в собственном соку и сыром.</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="15" hidden="0" customHeight="1">
@@ -24025,7 +24051,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C153" s="25" t="str">
-        <x:v>Добавь начинку и запекай ещё 10 минут.</x:v>
+        <x:v>Добавь томаты в собственном соку, моцареллу, курицу и овощи, запекай ещё 10 минут.</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="15" hidden="0" customHeight="1">
@@ -24102,7 +24128,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C160" s="25" t="str">
-        <x:v>Заверни фарш в баклажаны, залей томатным соусом, посыпь сыром и запеки 20 минут.</x:v>
+        <x:v>Заверни фарш в баклажаны, залей томатами в собственном соку, посыпь сыром и запеки 20 минут.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
@@ -24278,7 +24304,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C176" s="25" t="str">
-        <x:v>Заверни в тортильи, выложи в форму, залей томатным соусом, посыпь сыром и запеки 20 минут.</x:v>
+        <x:v>Заверни в тортильи, выложи в форму, залей томатами в собственном соку, посыпь сыром и запеки 20 минут.</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
@@ -25422,7 +25448,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C280" s="25" t="str">
-        <x:v>смажь лаваш соусом, добавь начинку и сыр.</x:v>
+        <x:v>Смажь лаваш томатами в собственном соку, добавь помидоры, оливки, базилик и сыр.</x:v>
       </x:c>
     </x:row>
     <x:row r="281" ht="15" hidden="0" customHeight="1">
@@ -25488,7 +25514,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C286" s="25" t="str">
-        <x:v>намажь хлеб соусом, добавь начинку и сыр.</x:v>
+        <x:v>Намажь хлеб томатами в собственном соку, добавь помидор, курицу и сыр.</x:v>
       </x:c>
     </x:row>
     <x:row r="287" ht="15" hidden="0" customHeight="1">
@@ -25567,10 +25593,10 @@
         <x:v>note</x:v>
       </x:c>
       <x:c r="C4" s="24" t="str">
-        <x:v>Белковый ингредиент 'плавленый сыр' не явно назван в шагах.</x:v>
+        <x:v>Белковый ингредиент 'творожный сыр' назван в шаге после rescue-fix.</x:v>
       </x:c>
       <x:c r="D4" s="25" t="str">
-        <x:v>При необходимости уточнить шаг, чтобы белковый ингредиент был назван явно.</x:v>
+        <x:v>No action; ingredient and step now align.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -26628,13 +26654,13 @@
         <x:v>batch2_052</x:v>
       </x:c>
       <x:c r="B80" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C80" s="24" t="str">
-        <x:v>В исходнике нет приема пищи и сложности; основной слот и effort восстановлены редакционно.</x:v>
+        <x:v>Rescue policy: main slot, interesting effort, and one-portion quantities accepted as conservative editorial correction.</x:v>
       </x:c>
       <x:c r="D80" s="25" t="str">
-        <x:v>Подтвердить слот, effort и порцию перед импортом.</x:v>
+        <x:v>No import blocker after tomato normalization; keep source-restoration note for audit trail.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
@@ -28294,13 +28320,13 @@
         <x:v>batch2_002</x:v>
       </x:c>
       <x:c r="B199" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C199" s="24" t="str">
-        <x:v>Prepared crab sticks require policy review; status set to needs_review.</x:v>
+        <x:v>Rescue policy: крабовые палочки map to canonical food_id crab_sticks; status set to ready without decomposition.</x:v>
       </x:c>
       <x:c r="D199" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may keep crab sticks as the canonical ingredient.</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="24" hidden="0" customHeight="1">
@@ -28308,13 +28334,13 @@
         <x:v>batch2_005</x:v>
       </x:c>
       <x:c r="B200" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C200" s="24" t="str">
-        <x:v>Prepared crab sticks and processed cheese require policy review; status set to needs_review.</x:v>
+        <x:v>Rescue policy: крабовые палочки map to canonical food_id crab_sticks; плавленый сыр replaced with творожный сыр; status set to ready.</x:v>
       </x:c>
       <x:c r="D200" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may keep crab sticks and use творожный сыр/cream_cheese mapping.</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="24" hidden="0" customHeight="1">
@@ -28322,13 +28348,13 @@
         <x:v>batch2_052</x:v>
       </x:c>
       <x:c r="B201" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C201" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; recipe stays needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; status set to ready.</x:v>
       </x:c>
       <x:c r="D201" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may use томаты в собственном соку; no prepared tomato sauce row remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="24" hidden="0" customHeight="1">
@@ -28336,13 +28362,13 @@
         <x:v>batch2_053</x:v>
       </x:c>
       <x:c r="B202" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C202" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; status set to needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; status set to ready.</x:v>
       </x:c>
       <x:c r="D202" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may use томаты в собственном соку; no prepared tomato sauce row remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="24" hidden="0" customHeight="1">
@@ -28350,13 +28376,13 @@
         <x:v>batch2_055</x:v>
       </x:c>
       <x:c r="B203" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C203" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; status set to needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; status set to ready.</x:v>
       </x:c>
       <x:c r="D203" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may use томаты в собственном соку; no prepared tomato sauce row remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="24" hidden="0" customHeight="1">
@@ -28364,13 +28390,13 @@
         <x:v>batch2_060</x:v>
       </x:c>
       <x:c r="B204" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C204" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; status set to needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; status set to ready.</x:v>
       </x:c>
       <x:c r="D204" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may use томаты в собственном соку; no prepared tomato sauce row remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="24" hidden="0" customHeight="1">
@@ -28381,10 +28407,10 @@
         <x:v>warning</x:v>
       </x:c>
       <x:c r="C205" s="24" t="str">
-        <x:v>Prepared canned sprats row remains; status set to needs_review pending policy decision.</x:v>
+        <x:v>Sprats remain needs_review: no production food_id for sprats or close canned fish mapping; drained-weight note added but import mapping is unsupported.</x:v>
       </x:c>
       <x:c r="D205" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Add or approve a canonical canned sprats food before import, or keep excluded from ready import.</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="24" hidden="0" customHeight="1">
@@ -28395,10 +28421,10 @@
         <x:v>warning</x:v>
       </x:c>
       <x:c r="C206" s="24" t="str">
-        <x:v>Prepared canned sprats row remains; status set to needs_review pending policy decision.</x:v>
+        <x:v>Sprats remain needs_review: no production food_id for sprats or close canned fish mapping; drained-weight note added but import mapping is unsupported.</x:v>
       </x:c>
       <x:c r="D206" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Add or approve a canonical canned sprats food before import, or keep excluded from ready import.</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="24" hidden="0" customHeight="1">
@@ -28409,10 +28435,10 @@
         <x:v>warning</x:v>
       </x:c>
       <x:c r="C207" s="24" t="str">
-        <x:v>Prepared canned sprats row remains; status set to needs_review pending policy decision.</x:v>
+        <x:v>Sprats remain needs_review: no production food_id for sprats or close canned fish mapping; drained-weight note added but import mapping is unsupported.</x:v>
       </x:c>
       <x:c r="D207" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Add or approve a canonical canned sprats food before import, or keep excluded from ready import.</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="24" hidden="0" customHeight="1">
@@ -28423,10 +28449,10 @@
         <x:v>warning</x:v>
       </x:c>
       <x:c r="C208" s="24" t="str">
-        <x:v>Prepared canned sprats row remains; status set to needs_review pending policy decision.</x:v>
+        <x:v>Sprats remain needs_review: no production food_id for sprats or close canned fish mapping; drained-weight note added but import mapping is unsupported.</x:v>
       </x:c>
       <x:c r="D208" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Add or approve a canonical canned sprats food before import, or keep excluded from ready import.</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="24" hidden="0" customHeight="1">
@@ -28434,13 +28460,13 @@
         <x:v>batch2_102</x:v>
       </x:c>
       <x:c r="B209" s="24" t="str">
-        <x:v>warning</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C209" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; status set to needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; status set to ready.</x:v>
       </x:c>
       <x:c r="D209" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Ready import may use томаты в собственном соку; no prepared tomato sauce row remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="24" hidden="0" customHeight="1">
@@ -28451,10 +28477,10 @@
         <x:v>warning</x:v>
       </x:c>
       <x:c r="C210" s="24" t="str">
-        <x:v>Prepared tomato sauce row remains; recipe stays needs_review until sauce is decomposed.</x:v>
+        <x:v>Rescue policy: томатный соус заменен на томаты в собственном соку, но source lacks exact one-portion quantities; recipe stays needs_review.</x:v>
       </x:c>
       <x:c r="D210" s="25" t="str">
-        <x:v>Do not import as ready until the prepared product is decomposed into policy-compliant ingredients or explicitly approved.</x:v>
+        <x:v>Confirm exact quantities before import; prepared tomato sauce itself is no longer the blocker.</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
recipes: resolve final second intake review recipe
</commit_message>
<xml_diff>
--- a/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
+++ b/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="recipes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ingredients" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="steps" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="qa_issues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ingredients" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="steps" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qa_issues" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="R107" s="28" t="inlineStr">
         <is>
-          <t>needs_review</t>
+          <t>ready</t>
         </is>
       </c>
     </row>
@@ -33080,7 +33080,7 @@
       </c>
       <c r="H683" s="25" t="inlineStr">
         <is>
-          <t>Количество восстановлено редакционно из названия/шага.</t>
+          <t>Manual rescue: 2 slices / 60 g matches ready hot sandwich pattern batch2_104.</t>
         </is>
       </c>
     </row>
@@ -33120,7 +33120,7 @@
       </c>
       <c r="H684" s="25" t="inlineStr">
         <is>
-          <t>Rescue policy: томатный соус заменен на томаты в собственном соку с тем же граммажем; рецепт остается needs_review из-за неточных source quantities.</t>
+          <t>Manual rescue: 120 g matches ready lazy pizza pattern batch2_102; prepared tomato sauce remains normalized.</t>
         </is>
       </c>
     </row>
@@ -33156,7 +33156,7 @@
       </c>
       <c r="H685" s="25" t="inlineStr">
         <is>
-          <t>Количество восстановлено редакционно из названия/шага.</t>
+          <t>Manual rescue: 30 g matches ready lazy pizza/hot sandwich pattern batch2_102/batch2_104.</t>
         </is>
       </c>
     </row>
@@ -33192,7 +33192,7 @@
       </c>
       <c r="H686" s="25" t="inlineStr">
         <is>
-          <t>Количество восстановлено редакционно из названия/шага.</t>
+          <t>Manual rescue: 120 g matches ready lazy pizza/hot sandwich pattern batch2_102/batch2_104.</t>
         </is>
       </c>
     </row>
@@ -33228,7 +33228,7 @@
       </c>
       <c r="H687" s="28" t="inlineStr">
         <is>
-          <t>Количество восстановлено редакционно из названия/шага.</t>
+          <t>Manual rescue: 90 g is within ready chicken sandwich/roll pattern range and is explicitly named in the step.</t>
         </is>
       </c>
     </row>
@@ -41815,12 +41815,12 @@
       </c>
       <c r="C193" s="24" t="inlineStr">
         <is>
-          <t>В исходнике не указан прием пищи.</t>
+          <t>Manual rescue: meal slot accepted as breakfast,snack by analogy with ready batch2_102 and batch2_104.</t>
         </is>
       </c>
       <c r="D193" s="25" t="inlineStr">
         <is>
-          <t>Проверить при production-import.</t>
+          <t>No further action before ready-only importer dry-run.</t>
         </is>
       </c>
     </row>
@@ -41837,12 +41837,12 @@
       </c>
       <c r="C194" s="24" t="inlineStr">
         <is>
-          <t>В исходнике не указана сложность.</t>
+          <t>Manual rescue: effort accepted as simple by analogy with ready 10-minute skillet bread/lavash recipes.</t>
         </is>
       </c>
       <c r="D194" s="25" t="inlineStr">
         <is>
-          <t>Проверить при production-import.</t>
+          <t>No further action before ready-only importer dry-run.</t>
         </is>
       </c>
     </row>
@@ -41854,17 +41854,17 @@
       </c>
       <c r="B195" s="24" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>note</t>
         </is>
       </c>
       <c r="C195" s="24" t="inlineStr">
         <is>
-          <t>В исходнике нет приема пищи, сложности и точных количеств; нужна ручная проверка перед production-import.</t>
+          <t>Manual rescue resolved: quantities, slot, effort, and skillet equipment align with ready pizza/sandwich patterns.</t>
         </is>
       </c>
       <c r="D195" s="25" t="inlineStr">
         <is>
-          <t>Подтвердить слот, effort и порцию перед импортом.</t>
+          <t>Ready for ready-only importer dry-run; do not import batch2_008.</t>
         </is>
       </c>
     </row>
@@ -41881,12 +41881,12 @@
       </c>
       <c r="C196" s="24" t="inlineStr">
         <is>
-          <t>5 количеств восстановлены редакционно из неполного исходника.</t>
+          <t>Manual rescue: five restored quantities accepted after comparison with ready batch2_102, batch2_104, and chicken sandwich rows.</t>
         </is>
       </c>
       <c r="D196" s="25" t="inlineStr">
         <is>
-          <t>Сверить граммовки при ручном QA.</t>
+          <t>Keep the documented gram estimates.</t>
         </is>
       </c>
     </row>
@@ -41903,12 +41903,12 @@
       </c>
       <c r="C197" s="24" t="inlineStr">
         <is>
-          <t>Белковый ингредиент 'курица' не явно назван в шагах.</t>
+          <t>Manual rescue: step 1 explicitly names chicken after tomato/pizza wording normalization.</t>
         </is>
       </c>
       <c r="D197" s="25" t="inlineStr">
         <is>
-          <t>При необходимости уточнить шаг, чтобы белковый ингредиент был назван явно.</t>
+          <t>No step change required.</t>
         </is>
       </c>
     </row>
@@ -42184,17 +42184,17 @@
       </c>
       <c r="B210" s="24" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>note</t>
         </is>
       </c>
       <c r="C210" s="24" t="inlineStr">
         <is>
-          <t>Rescue policy: томатный соус заменен на томаты в собственном соку, но source lacks exact one-portion quantities; recipe stays needs_review.</t>
+          <t>Manual rescue resolved: tomato sauce normalization matches ready batch2_102, and the recipe is ready with tomatoes in own juice.</t>
         </is>
       </c>
       <c r="D210" s="25" t="inlineStr">
         <is>
-          <t>Confirm exact quantities before import; prepared tomato sauce itself is no longer the blocker.</t>
+          <t>Ready for ready-only importer dry-run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
recipes: complete under-composed main dishes
</commit_message>
<xml_diff>
--- a/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
+++ b/tmp/recipe_intake_batch2/cleaned_recipes_batch2.xlsx
@@ -9946,22 +9946,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>хлеба</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>цельнозерновой хлеб</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>60</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ломтика</t>
-        </is>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>60</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Data repair batch 1: two bread slices restored as 60 g.</t>
         </is>
       </c>
     </row>
@@ -11721,22 +11727,28 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>цельнозернового хлеба</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>цельнозерновой хлеб</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>60</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>ломтика</t>
-        </is>
+          <t>г</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>60</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Data repair batch 1: two bread slices restored as 60 g.</t>
         </is>
       </c>
     </row>
@@ -19110,22 +19122,25 @@
           <t>рис</t>
         </is>
       </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>0,5</t>
-        </is>
+      <c r="C296" t="n">
+        <v>60</v>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>ст. л.</t>
+          <t>г</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="G296" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Data repair batch 1: rice side restored.</t>
         </is>
       </c>
     </row>
@@ -33765,7 +33780,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Подсушите хлеб на сухой сковороде, натрите чесноком и сбрызните оливковым маслом.</t>
+          <t>Подсушите два ломтика цельнозернового хлеба на сухой сковороде, натрите чесноком и сбрызните оливковым маслом.</t>
         </is>
       </c>
     </row>
@@ -34110,7 +34125,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Смажьте два ломтика хлеба йогуртом со специями, выложите салатные листья, курицу, кружочки помидора и сыр.</t>
+          <t>Смажьте два ломтика цельнозернового хлеба йогуртом со специями, выложите салатные листья, курицу, кружочки помидора и сыр.</t>
         </is>
       </c>
     </row>
@@ -34125,7 +34140,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Накройте сэндвичи оставшимся хлебом.</t>
+          <t>Накройте сэндвич оставшимся хлебом.</t>
         </is>
       </c>
     </row>
@@ -35355,7 +35370,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Подавайте с вареным рисом.</t>
+          <t>Отварите рис до готовности и подавайте с куриным карри.</t>
         </is>
       </c>
     </row>

</xml_diff>